<commit_message>
Add 13 additional works by António Lobo Antunes
- Expanded António Lobo Antunes collection from 4 to 17 works
- Added major novels: Acto de Condenação, Manual dos Inquisidores, O Filho da Mãe, Não Morrer, and others
- Total catalog now: 159 works from 15 authors
- Years covered: 1979-2011 for this author

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J3QcMLUcYVgwk3FeRRMBWq
</commit_message>
<xml_diff>
--- a/CATALOGO_MEGA_COMPLETO_2026.xlsx
+++ b/CATALOGO_MEGA_COMPLETO_2026.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G147"/>
+  <dimension ref="A1:G160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5507,6 +5507,461 @@
         <v>15</v>
       </c>
     </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>António Lobo Antunes</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Acto de Condenação</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>1990</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Livros do Brasil</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Disponível</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>António Lobo Antunes</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>A Ordem Natural das Coisas</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>1992</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Livros do Brasil</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Disponível</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>António Lobo Antunes</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Manual dos Inquisidores</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>1996</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Livros do Brasil</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Disponível</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>António Lobo Antunes</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Exortação aos Crocodilos</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>1999</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Livros do Brasil</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Disponível</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>António Lobo Antunes</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>A Primeira Noite do Resto da Tua Vida</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Livros do Brasil</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Disponível</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>António Lobo Antunes</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>A Alga</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>2004</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Livros do Brasil</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Disponível</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>António Lobo Antunes</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>A Clemência dos Reis</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>2005</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Livros do Brasil</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Disponível</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>António Lobo Antunes</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Com Raiva, Piedade e Covardia</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>2007</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Livros do Brasil</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Disponível</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>António Lobo Antunes</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Não Morrer</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>2008</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Livros do Brasil</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Disponível</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>António Lobo Antunes</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Adão e Eva</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>2010</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Livros do Brasil</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Disponível</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>António Lobo Antunes</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>As Preces e os Gestos</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>2011</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Livros do Brasil</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Disponível</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>António Lobo Antunes</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>O Filho da Mãe</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>2007</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Livros do Brasil</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Disponível</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>António Lobo Antunes</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>A Comichão da Asa Esquerda</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>2008</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Livros do Brasil</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Disponível</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Romance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>